<commit_message>
Change entity models, add erd
</commit_message>
<xml_diff>
--- a/docs/Data architecture/Entities/ClientBlock.xlsx
+++ b/docs/Data architecture/Entities/ClientBlock.xlsx
@@ -5,18 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Computer Science\Programming\C#\Projects\RealProjects\NeUrokAdmin\docs\Data architecture\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Computer Science\Programming\C#\Projects\RealProjects\NeUrokAdmin\docs\Data architecture\Entities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828DE21F-F906-4A3B-ACA3-BEDD6F852C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98A4A13-6050-49E0-9010-DED718F0AE22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28710" yWindow="-90" windowWidth="28980" windowHeight="16380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4080" yWindow="1005" windowWidth="23805" windowHeight="13440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="clients" sheetId="1" r:id="rId1"/>
-    <sheet name="courses" sheetId="3" r:id="rId2"/>
-    <sheet name="client_statuses" sheetId="2" r:id="rId3"/>
-    <sheet name="client_courses" sheetId="4" r:id="rId4"/>
+    <sheet name="users" sheetId="5" r:id="rId1"/>
+    <sheet name="clients" sheetId="1" r:id="rId2"/>
+    <sheet name="courses" sheetId="3" r:id="rId3"/>
+    <sheet name="client_statuses" sheetId="2" r:id="rId4"/>
+    <sheet name="client_courses" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="80">
   <si>
     <t>Бегунова Дарья Алексеевна</t>
   </si>
@@ -201,9 +202,6 @@
     <t>phone</t>
   </si>
   <si>
-    <t>comments</t>
-  </si>
-  <si>
     <t>additional_phones</t>
   </si>
   <si>
@@ -259,6 +257,18 @@
   </si>
   <si>
     <t>course_id</t>
+  </si>
+  <si>
+    <t>login</t>
+  </si>
+  <si>
+    <t>password_hash</t>
+  </si>
+  <si>
+    <t>password_salt</t>
+  </si>
+  <si>
+    <t>notes</t>
   </si>
 </sst>
 </file>
@@ -612,6 +622,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75867046-7733-4E9E-96EC-CD046E19AE76}">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -637,13 +674,13 @@
         <v>53</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>61</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>54</v>
@@ -655,10 +692,10 @@
         <v>56</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -1266,7 +1303,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{857B95D0-73A1-439A-A671-17F57FA7831A}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1280,7 +1317,7 @@
         <v>52</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1288,7 +1325,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1296,7 +1333,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1304,7 +1341,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1312,7 +1349,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1320,7 +1357,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1336,7 +1373,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B09E5D5-7014-4A90-9B26-AA9FBCF73EB6}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1350,7 +1387,7 @@
         <v>52</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1358,7 +1395,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1366,7 +1403,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1374,7 +1411,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1382,7 +1419,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1390,7 +1427,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1398,7 +1435,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1406,17 +1443,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECA056FE-E0CB-4B7E-8169-F6D34379D635}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>